<commit_message>
Compact countdown, task sorting, Ezraider 15% discount, refreshed downloads
- Countdown: compact inline line under hero subtitle; switches to return flight after outbound departs, hides after return
- Tasks: completed tasks sink to the bottom (ordered by completion time)
- Ezraider pricing: per-vehicle (70€ driver / 35€ passenger), 9 vehicles, 15% discount → ~654.50€ total
- Updated cost summaries to reflect the discount
- Refresh athens_full_plan.pdf and athens_trip_full.xlsx

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/downloads/athens_trip_full.xlsx
+++ b/public/downloads/athens_trip_full.xlsx
@@ -877,7 +877,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>נקודת מפגש לתיאום</t>
+          <t>Leof. Andrea Siggrou 22 — GoGo Electric</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>לאשר יציאה ב-14:45 + נגישות לסבתא!</t>
+          <t>🚖 לקחת אובר! לאשר יציאה ב-14:45 + נגישות לסבתא</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>70€ מבוגר / 35€ ילד</t>
+          <t>59.50€ מבוגר / 29.75€ ילד</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2195,7 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>70 euro מבוגר / 35 euro ילד. לאשר יציאה ב-14:45 + נגישות לסבתא</t>
+          <t>59.50 euro מבוגר / 29.75 euro ילד (15% הנחה). לאשר יציאה ב-14:45 + נגישות לסבתא</t>
         </is>
       </c>
     </row>
@@ -2672,16 +2672,16 @@
         </is>
       </c>
       <c r="B13" s="11" t="n">
-        <v>70</v>
+        <v>59.5</v>
       </c>
       <c r="C13" s="11" t="n">
-        <v>35</v>
+        <v>29.75</v>
       </c>
       <c r="D13" s="11" t="n">
-        <v>251</v>
+        <v>213</v>
       </c>
       <c r="E13" s="11" t="n">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="F13" s="11" t="n">
         <v>9</v>
@@ -2691,12 +2691,12 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>~770</t>
+          <t>~655</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>מחיר קבוע לאדם</t>
+          <t>15% הנחה. מחיר מקורי 70/35€</t>
         </is>
       </c>
     </row>
@@ -4175,12 +4175,12 @@
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>לאשר ב-14:45 + נגישות לסבתא.</t>
+          <t>🚖 אובר ל-Leof. Andrea Siggrou 22. לאשר ב-14:45.</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
         <is>
-          <t>70€ מבוגר / 35€ ילד</t>
+          <t>59.50€ מבוגר / 29.75€ ילד (15% הנחה)</t>
         </is>
       </c>
       <c r="F10" s="23" t="inlineStr">

</xml_diff>

<commit_message>
fix: update travel times and hotel details for Titania Hotel
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/public/downloads/athens_trip_full.xlsx
+++ b/public/downloads/athens_trip_full.xlsx
@@ -748,7 +748,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel - Diomeias 5</t>
+          <t>Titania Hotel Athens</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -971,7 +971,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel</t>
+          <t>Titania Hotel Athens</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -1327,7 +1327,7 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel</t>
+          <t>Titania Hotel Athens</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel</t>
+          <t>Titania Hotel Athens</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr"/>
@@ -1933,7 +1933,7 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel</t>
+          <t>Titania Hotel Athens</t>
         </is>
       </c>
       <c r="F30" s="6" t="inlineStr"/>
@@ -2244,7 +2244,7 @@
       <c r="B9" s="7" t="inlineStr"/>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>Athens Cypria Hotel - Diomeias 5</t>
+          <t>Titania Hotel Athens - Diomeias 5</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr"/>
@@ -2261,7 +2261,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2551,215 +2551,201 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>מלון — 4 חדרים 3 לילות (Agoda)</t>
+          <t>מלון — הזמנה 1 (59110948) 5 חדרים</t>
         </is>
       </c>
       <c r="B10" s="10" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="C10" s="10" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" s="10" t="n">
-        <v>4</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="G10" s="10" t="inlineStr"/>
       <c r="H10" s="10" t="n">
-        <v>2064.44</v>
+        <v>1725</v>
       </c>
       <c r="I10" s="10" t="inlineStr">
         <is>
-          <t>תשלום אוטומטי 19 אפריל!</t>
+          <t>כולל ארוחת בוקר. Climate Tax 150€ בצ'ק-אין</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>הסעה שדה + מלון (x2)</t>
-        </is>
-      </c>
-      <c r="B11" s="11" t="inlineStr">
-        <is>
-          <t>~23</t>
-        </is>
-      </c>
-      <c r="C11" s="11" t="inlineStr">
-        <is>
-          <t>~23</t>
-        </is>
-      </c>
-      <c r="D11" s="11" t="inlineStr">
-        <is>
-          <t>~82</t>
-        </is>
-      </c>
-      <c r="E11" s="11" t="inlineStr">
-        <is>
-          <t>~82</t>
-        </is>
-      </c>
-      <c r="F11" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="G11" s="11" t="inlineStr"/>
-      <c r="H11" s="11" t="inlineStr">
-        <is>
-          <t>~300</t>
-        </is>
-      </c>
-      <c r="I11" s="11" t="inlineStr">
-        <is>
-          <t>150€ לכיוון × 2 ÷ 13</t>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>מלון — הזמנה 2 (59110949) 1 חדר</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="D11" s="10" t="n">
+        <v>408</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>408</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="10" t="inlineStr"/>
+      <c r="H11" s="10" t="n">
+        <v>345</v>
+      </c>
+      <c r="I11" s="10" t="inlineStr">
+        <is>
+          <t>אדיר+הילה+כפיר. Climate Tax 30€ בצ'ק-אין</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="11" t="inlineStr">
         <is>
-          <t>הופ-און הופ-אוף</t>
+          <t>הסעה שדה + מלון (x2)</t>
         </is>
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>~28</t>
+          <t>~23</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>~14</t>
+          <t>~23</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>~100</t>
+          <t>~82</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">
         <is>
-          <t>~50</t>
+          <t>~82</t>
         </is>
       </c>
       <c r="F12" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>4</v>
-      </c>
+        <v>13</v>
+      </c>
+      <c r="G12" s="11" t="inlineStr"/>
       <c r="H12" s="11" t="inlineStr">
         <is>
-          <t>~280</t>
+          <t>~300</t>
         </is>
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>כרטיס 48 שעות</t>
+          <t>150€ לכיוון × 2 ÷ 13</t>
         </is>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>סיור Ezraider</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n">
-        <v>59.5</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <v>29.75</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>213</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>106</v>
+          <t>הופ-און הופ-אוף</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>~28</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>~14</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>~100</t>
+        </is>
+      </c>
+      <c r="E13" s="11" t="inlineStr">
+        <is>
+          <t>~50</t>
+        </is>
       </c>
       <c r="F13" s="11" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G13" s="11" t="n">
         <v>4</v>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>~655</t>
+          <t>~280</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>15% הנחה. מחיר מקורי 70/35€</t>
+          <t>כרטיס 48 שעות</t>
         </is>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="11" t="inlineStr">
         <is>
-          <t>Who Killed Callimachos</t>
+          <t>סיור Ezraider</t>
         </is>
       </c>
       <c r="B14" s="11" t="n">
-        <v>22</v>
+        <v>59.5</v>
       </c>
       <c r="C14" s="11" t="n">
-        <v>15</v>
+        <v>29.75</v>
       </c>
       <c r="D14" s="11" t="n">
-        <v>79</v>
+        <v>213</v>
       </c>
       <c r="E14" s="11" t="n">
-        <v>54</v>
+        <v>106</v>
       </c>
       <c r="F14" s="11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G14" s="11" t="n">
         <v>4</v>
       </c>
       <c r="H14" s="11" t="inlineStr">
         <is>
-          <t>~236</t>
+          <t>~655</t>
         </is>
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>הנחה קבוצתית ל-10+</t>
+          <t>15% הנחה. מחיר מקורי 70/35€</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>טיול יום — נפפליאו (ואן פרטי)</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>~54</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>~54</t>
-        </is>
-      </c>
-      <c r="D15" s="11" t="inlineStr">
-        <is>
-          <t>~193</t>
-        </is>
-      </c>
-      <c r="E15" s="11" t="inlineStr">
-        <is>
-          <t>~193</t>
-        </is>
+          <t>Who Killed Callimachos</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="n">
+        <v>22</v>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="D15" s="11" t="n">
+        <v>79</v>
+      </c>
+      <c r="E15" s="11" t="n">
+        <v>54</v>
       </c>
       <c r="F15" s="11" t="n">
         <v>8</v>
@@ -2767,39 +2753,41 @@
       <c r="G15" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H15" s="11" t="n">
-        <v>650</v>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>~236</t>
+        </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>650 euro / 12. כולל תעלת קורינטוס</t>
+          <t>הנחה קבוצתית ל-10+</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>כניסה מבצר פלמידי</t>
+          <t>טיול יום — נפפליאו (ואן פרטי)</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>~8</t>
+          <t>~54</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>~8</t>
+          <t>~54</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>~29</t>
+          <t>~193</t>
         </is>
       </c>
       <c r="E16" s="11" t="inlineStr">
         <is>
-          <t>~29</t>
+          <t>~193</t>
         </is>
       </c>
       <c r="F16" s="11" t="n">
@@ -2808,34 +2796,40 @@
       <c r="G16" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H16" s="11" t="inlineStr">
-        <is>
-          <t>~96</t>
-        </is>
+      <c r="H16" s="11" t="n">
+        <v>650</v>
       </c>
       <c r="I16" s="11" t="inlineStr">
         <is>
-          <t>ילדים עד 18 — חינם</t>
+          <t>650 euro / 12. כולל תעלת קורינטוס</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>גבעת ליקבטוס (רכבל)</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="C17" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="D17" s="11" t="n">
-        <v>47</v>
-      </c>
-      <c r="E17" s="11" t="n">
-        <v>47</v>
+          <t>כניסה מבצר פלמידי</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>~8</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>~29</t>
+        </is>
+      </c>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>~29</t>
+        </is>
       </c>
       <c r="F17" s="11" t="n">
         <v>8</v>
@@ -2845,40 +2839,32 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>~156</t>
+          <t>~96</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>הלוך-חזור</t>
+          <t>ילדים עד 18 — חינם</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
-          <t>מוזיאון האשליות</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
-        <is>
-          <t>~13</t>
-        </is>
-      </c>
-      <c r="C18" s="11" t="inlineStr">
-        <is>
-          <t>~13</t>
-        </is>
-      </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>~47</t>
-        </is>
-      </c>
-      <c r="E18" s="11" t="inlineStr">
-        <is>
-          <t>~47</t>
-        </is>
+          <t>גבעת ליקבטוס (רכבל)</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="C18" s="11" t="n">
+        <v>13</v>
+      </c>
+      <c r="D18" s="11" t="n">
+        <v>47</v>
+      </c>
+      <c r="E18" s="11" t="n">
+        <v>47</v>
       </c>
       <c r="F18" s="11" t="n">
         <v>8</v>
@@ -2893,34 +2879,34 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>הנחות קבוצה — לשאול</t>
+          <t>הלוך-חזור</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="11" t="inlineStr">
         <is>
-          <t>ארוחות צהריים x4</t>
+          <t>מוזיאון האשליות</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>~22</t>
+          <t>~13</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>~15</t>
+          <t>~13</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>~79</t>
+          <t>~47</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
         <is>
-          <t>~54</t>
+          <t>~47</t>
         </is>
       </c>
       <c r="F19" s="11" t="n">
@@ -2931,98 +2917,114 @@
       </c>
       <c r="H19" s="11" t="inlineStr">
         <is>
-          <t>~816</t>
+          <t>~156</t>
         </is>
       </c>
       <c r="I19" s="11" t="inlineStr">
         <is>
-          <t>ממוצע</t>
+          <t>הנחות קבוצה — לשאול</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
+          <t>ארוחות צהריים x4</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>~22</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>~15</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>~79</t>
+        </is>
+      </c>
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>~54</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="G20" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="H20" s="11" t="inlineStr">
+        <is>
+          <t>~816</t>
+        </is>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>ממוצע</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>קניות / קפה / שונות</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>~30</t>
         </is>
       </c>
-      <c r="C20" s="11" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>~30</t>
         </is>
       </c>
-      <c r="D20" s="11" t="inlineStr">
+      <c r="D21" s="11" t="inlineStr">
         <is>
           <t>~107</t>
         </is>
       </c>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>~107</t>
         </is>
       </c>
-      <c r="F20" s="11" t="n">
+      <c r="F21" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="G20" s="11" t="inlineStr"/>
-      <c r="H20" s="11" t="inlineStr">
+      <c r="G21" s="11" t="inlineStr"/>
+      <c r="H21" s="11" t="inlineStr">
         <is>
           <t>~360</t>
         </is>
       </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="I21" s="11" t="inlineStr">
         <is>
           <t>לפי שיקול דעת אישי</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>סה"כ פעילויות+אוכל — מבוגר</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>~270-320</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr"/>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>~967-1146</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="inlineStr"/>
-      <c r="F21" s="12" t="inlineStr"/>
-      <c r="G21" s="12" t="inlineStr"/>
-      <c r="H21" s="12" t="inlineStr"/>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>לא כולל קניות אישיות</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="12" t="inlineStr">
         <is>
-          <t>סה"כ פעילויות+אוכל — ילד/נוער</t>
+          <t>סה"כ פעילויות+אוכל — מבוגר</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
         <is>
-          <t>~193-233</t>
+          <t>~270-320</t>
         </is>
       </c>
       <c r="C22" s="12" t="inlineStr"/>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>~691-834</t>
+          <t>~967-1146</t>
         </is>
       </c>
       <c r="E22" s="12" t="inlineStr"/>
@@ -3031,25 +3033,25 @@
       <c r="H22" s="12" t="inlineStr"/>
       <c r="I22" s="12" t="inlineStr">
         <is>
-          <t>הנחות כניסה / פחות אוכל</t>
+          <t>לא כולל קניות אישיות</t>
         </is>
       </c>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>סה"כ כולל הכל — מבוגר (בסיס)</t>
+          <t>סה"כ פעילויות+אוכל — ילד/נוער</t>
         </is>
       </c>
       <c r="B23" s="12" t="inlineStr">
         <is>
-          <t>~599</t>
+          <t>~193-233</t>
         </is>
       </c>
       <c r="C23" s="12" t="inlineStr"/>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>~2,144</t>
+          <t>~691-834</t>
         </is>
       </c>
       <c r="E23" s="12" t="inlineStr"/>
@@ -3058,25 +3060,25 @@
       <c r="H23" s="12" t="inlineStr"/>
       <c r="I23" s="12" t="inlineStr">
         <is>
-          <t>שער 3.58 ILS/euro (15/4/2026)</t>
+          <t>הנחות כניסה / פחות אוכל</t>
         </is>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>סה"כ כולל הכל — ילד/נוער</t>
+          <t>סה"כ כולל הכל — מבוגר (בסיס)</t>
         </is>
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>~517</t>
+          <t>~599</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr"/>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>~1,851</t>
+          <t>~2,144</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr"/>
@@ -3084,6 +3086,33 @@
       <c r="G24" s="12" t="inlineStr"/>
       <c r="H24" s="12" t="inlineStr"/>
       <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>שער 3.58 ILS/euro (15/4/2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>סה"כ כולל הכל — ילד/נוער</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>~517</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr"/>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>~1,851</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr"/>
+      <c r="F25" s="12" t="inlineStr"/>
+      <c r="G25" s="12" t="inlineStr"/>
+      <c r="H25" s="12" t="inlineStr"/>
+      <c r="I25" s="12" t="inlineStr">
         <is>
           <t>שער 3.58 ILS/euro (15/4/2026)</t>
         </is>
@@ -3194,10 +3223,10 @@
         <v>131.59</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
@@ -3233,10 +3262,10 @@
         <v>131.59</v>
       </c>
       <c r="H3" s="13" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I3" s="13" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
@@ -3272,10 +3301,10 @@
         <v>131.59</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
@@ -3311,10 +3340,10 @@
         <v>131.59</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
@@ -3350,10 +3379,10 @@
         <v>131.59</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
@@ -3389,10 +3418,10 @@
         <v>213.59</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>172.04</v>
+        <v>115</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>385.63</v>
+        <v>328.59</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
@@ -3428,10 +3457,10 @@
         <v>131.59</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
@@ -3467,10 +3496,10 @@
         <v>195.59</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>367.63</v>
+        <v>368.09</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
@@ -3506,10 +3535,10 @@
         <v>195.59</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>367.63</v>
+        <v>368.09</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
@@ -3545,10 +3574,10 @@
         <v>145.59</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>172.04</v>
+        <v>115</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>317.63</v>
+        <v>260.59</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
@@ -3584,10 +3613,10 @@
         <v>145.59</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>172.04</v>
+        <v>115</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>317.63</v>
+        <v>260.59</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
@@ -3623,10 +3652,10 @@
         <v>213.59</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>385.63</v>
+        <v>386.09</v>
       </c>
     </row>
     <row r="14" ht="20" customHeight="1">
@@ -3662,10 +3691,10 @@
         <v>131.59</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>172.04</v>
+        <v>172.5</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>303.63</v>
+        <v>304.09</v>
       </c>
     </row>
   </sheetData>

</xml_diff>